<commit_message>
Ajouts N surplus et water 3.9
</commit_message>
<xml_diff>
--- a/data/3.10.2/2019_France/extensions/dom_biogeochemical/detail_levels.xlsx
+++ b/data/3.10.2/2019_France/extensions/dom_biogeochemical/detail_levels.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,42 +462,21 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>N - waste - water</t>
+          <t>N2O - agriculture - air</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>P - waste - water</t>
+          <t>NH3 - agriculture - air</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>NH3 - combustion - air</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>NH3 - non combustion - N- fertilizer production - air</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>NH3 - agriculture - air</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>NH3 - waste - air</t>
+          <t>NOX - agriculture - air</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ajout seuil et amélioration figure
</commit_message>
<xml_diff>
--- a/data/3.10.2/2019_France/extensions/dom_biogeochemical/detail_levels.xlsx
+++ b/data/3.10.2/2019_France/extensions/dom_biogeochemical/detail_levels.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,42 +441,399 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>N - agriculture - water</t>
+          <t>NH3 - combustion - air</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>P - agriculture - soil</t>
+          <t>NOx - combustion - air</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>P - agriculture - water</t>
+          <t>SO2 - combustion - air</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>N2O - agriculture - air</t>
+          <t>SOx - combustion - air</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>NH3 - agriculture - air</t>
+          <t>NH3 - non combustion - N- fertilizer production - air</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>NOx - non combustion - Agglomeration plant - pellets - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>NOx - non combustion - Agglomeration plant - sinter - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>NOx - non combustion - Bricks production - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>NOx - non combustion - Cement production - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>NOx - non combustion - Chemical wood pulp, dissolving grades - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>NOx - non combustion - Chemical wood pulp, soda and sulphate, other than dissolving grades - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>NOx - non combustion - Chemical wood pulp, sulphite, other than dissolving grades - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>NOx - non combustion - Glass production - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>NOx - non combustion - Lime production - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>NOx - non combustion - Nickel, unwrought - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>NOx - non combustion - Oil refinery - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>NOx - non combustion - Pig iron production, blast furnace - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>NOx - non combustion - Production of coke oven coke - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>NOx - non combustion - Production of gascoke - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>NOx - non combustion - Refined copper; unwrought, not alloyed - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>NOx - non combustion - Refined lead, unwrought - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>NOx - non combustion - Semi-chemical wood pulp, pulp of fibers other than wood - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>NOx - non combustion - Steel production: basic oxygen furnace - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>NOx - non combustion - Steel production: electric arc furnace - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>NOx - non combustion - Sulphuric acid production - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>NOx - non combustion - Unrefined copper; copper anodes for electrolytic refining - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>NOx - non combustion - Zinc, unwrought, not alloyed - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>SOx - non combustion - Agglomeration plant - sinter - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>SOx - non combustion - Bricks production - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>SOx - non combustion - Cement production - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>SOx - non combustion - Chemical wood pulp, dissolving grades - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>SOx - non combustion - Chemical wood pulp, soda and sulphate, other than dissolving grades - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>SOx - non combustion - Chemical wood pulp, sulphite, other than dissolving grades - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>SOx - non combustion - Glass production - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>SOx - non combustion - Lime production - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>SOx - non combustion - Nickel, unwrought - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>SOx - non combustion - Oil refinery - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>SOx - non combustion - Pig iron production, blast furnace - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>SOx - non combustion - Production of coke oven coke - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>SOx - non combustion - Production of gascoke - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>SOx - non combustion - Refined copper; unwrought, not alloyed - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>SOx - non combustion - Refined lead, unwrought - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>SOx - non combustion - Semi-chemical wood pulp, pulp of fibers other than wood - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>SOx - non combustion - Sulphuric acid production - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>SOx - non combustion - Unrefined copper; copper anodes for electrolytic refining - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>SOx - non combustion - Zinc, unwrought, not alloyed - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>N2O - agriculture - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>NH3 - agriculture - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
           <t>NOX - agriculture - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>NH3 - waste - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>NOX - waste - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>SOx - waste - air</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>N - agriculture - water</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>P - agriculture - soil</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>P - agriculture - water</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>N - waste - water</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>P - waste - water</t>
         </is>
       </c>
     </row>

</xml_diff>